<commit_message>
Update AutoTache persistent state
</commit_message>
<xml_diff>
--- a/cloud_state/offres_suivi.xlsx
+++ b/cloud_state/offres_suivi.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offres" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Offres'!$A$1:$AB$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Offres'!$A$1:$AB$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB37"/>
+  <dimension ref="A1:AB38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -4284,8 +4284,114 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-13T13:22:33</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ZzBsMlNKZTBmNkMweXY5VkFBQUFBQT09OkVzd0JDb3dCUVVwcFZEUjBTMEZ5UWtwdVZGZGtabnBDT0c1RWNqWlNWbWxXUm5WWloyOTBiRTU1U2tSdWJFeHVYMWhJUzFSeE5VVlNWbmRRYURSTFNuUkJXVWxpVkV0aGNsVXdXVGM1YmpOZk5raHROemxHYVZFNFQxaHJVbTB6TkVGcFZVOU5jVjh5YVZkRWJWaHpVV2M0WDNaZmFYRlpPWEpUTUZCeVRIUm5hRTFGWWxwNVZFbEVOSE5qWlRKVFdUTVNGMncyVDIxaGRYcHpSblY2U0hBNE5GQTFPRzFHTmtGUkdpSkJSSE55T1daVVYybzVXak41YVZad2VIRnVlVXRDZEc5RFozbGxSbkJHWWxWMw</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>JSearch</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Tech Lead Front End / Design System (F/H)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>BPCE Solutions informatiques</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Dijon, FR</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>À plein temps</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>teletravail partiel</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>HTML, CSS, JavaScript, React, Vue.js, Figma, UI, UX</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>2026-08-23T00:00:00.000Z</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Offre rejetee: devops pur.</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>À vérifier</t>
+        </is>
+      </c>
+      <c r="W38" t="n">
+        <v>55</v>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>À vérifier: score 55/100 grâce à technologies: frontend, figma, html, css, javascript, react, vue.js, design, design system, web, interface, maquette, accessibilite; titre: front end; domaine_metier: frontend, front end, ui, ux, design, maquette, interface; localisation: dijon; teletravail: teletravail.</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>technologies=35; titre=15; domaine_metier=15; localisation=15; teletravail=10; contrat=0; penalites=35</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>HTML, CSS, JavaScript, React, Vue.js, Figma</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>devops pur</t>
+        </is>
+      </c>
+      <c r="AB38" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/tech-lead-front-end-design-system-f-h-at-bpce-solutions-informatiques-4378935390</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB37"/>
+  <autoFilter ref="A1:AB38"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId2"/>
@@ -4323,6 +4429,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>